<commit_message>
add import First n Cells infos
</commit_message>
<xml_diff>
--- a/2-Tests/OpenExcelSdk.Tests/10-Files/SetCellColor.xlsx
+++ b/2-Tests/OpenExcelSdk.Tests/10-Files/SetCellColor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/2-Tests/OpenExcelSdk.Tests/10-Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56FEF93A-F737-4D83-B97F-C904CC996AC5}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A86D316-2893-4754-8652-6068E85DBDC6}"/>
   <bookViews>
-    <workbookView xWindow="4425" yWindow="4485" windowWidth="19065" windowHeight="9735" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
+    <workbookView xWindow="3270" yWindow="5835" windowWidth="19065" windowHeight="9735" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>cell</t>
   </si>
@@ -59,9 +59,6 @@
     <t>blue, set to yellow</t>
   </si>
   <si>
-    <t>gree, to to red</t>
-  </si>
-  <si>
     <t>null, set to yellow</t>
   </si>
   <si>
@@ -69,6 +66,18 @@
   </si>
   <si>
     <t>nofill, border, set to orange</t>
+  </si>
+  <si>
+    <t>later</t>
+  </si>
+  <si>
+    <t>green, to to red</t>
+  </si>
+  <si>
+    <t>pb</t>
+  </si>
+  <si>
+    <t>test</t>
   </si>
 </sst>
 </file>
@@ -110,7 +119,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -118,31 +127,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -158,10 +151,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -481,13 +470,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80C34316-5981-45DA-B1A5-D1338D5ADA96}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -495,7 +484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -503,35 +492,43 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4"/>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix numberFormat for account, built-in=44
</commit_message>
<xml_diff>
--- a/2-Tests/OpenExcelSdk.Tests/10-Files/SetCellColor.xlsx
+++ b/2-Tests/OpenExcelSdk.Tests/10-Files/SetCellColor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/2-Tests/OpenExcelSdk.Tests/10-Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A86D316-2893-4754-8652-6068E85DBDC6}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="8_{56AC0E10-4E35-4625-96F0-822C42176BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DCC025D-35BD-48AF-8EF9-1D1F44628FE6}"/>
   <bookViews>
-    <workbookView xWindow="3270" yWindow="5835" windowWidth="19065" windowHeight="9735" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
+    <workbookView xWindow="1410" yWindow="1815" windowWidth="23925" windowHeight="13350" xr2:uid="{E5BB3879-E844-49FA-BF0E-81D626AAA851}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>cell</t>
   </si>
@@ -68,13 +68,7 @@
     <t>nofill, border, set to orange</t>
   </si>
   <si>
-    <t>later</t>
-  </si>
-  <si>
     <t>green, to to red</t>
-  </si>
-  <si>
-    <t>pb</t>
   </si>
   <si>
     <t>test</t>
@@ -119,7 +113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -127,15 +121,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -151,6 +161,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -470,13 +484,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80C34316-5981-45DA-B1A5-D1338D5ADA96}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -484,7 +498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -492,44 +506,39 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4"/>
       <c r="B7" t="s">
         <v>9</v>
-      </c>
-      <c r="D7" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>